<commit_message>
Planilha de controle só com valores, pronta para copiar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/controle.xlsx
+++ b/controle.xlsx
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerada pelo script gerar_controle.py a partir do pessoas.json. Status = Concluído quando tem capa, versículo em todas as fotos e pelo menos 1 áudio.</t>
+          <t>Atualizada em 26/10/2026 pelo script gerar_controle.py. Status = Concluído quando tem capa, versículo em todas as fotos e pelo menos 1 áudio.</t>
         </is>
       </c>
     </row>
@@ -523,9 +523,8 @@
           <t>Concluídos</t>
         </is>
       </c>
-      <c r="B4" s="4">
-        <f>COUNTIF(C8:C200,"Concluído")</f>
-        <v/>
+      <c r="B4" s="4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -534,9 +533,8 @@
           <t>Pendentes</t>
         </is>
       </c>
-      <c r="B5" s="4">
-        <f>COUNTIF(C8:C200,"Pendente")</f>
-        <v/>
+      <c r="B5" s="4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -602,9 +600,10 @@
           <t>Catarina</t>
         </is>
       </c>
-      <c r="C8" s="7">
-        <f>IF(AND(D8="Sim",E8&gt;0,F8=E8,G8&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
@@ -643,9 +642,10 @@
           <t>Esther Caraça</t>
         </is>
       </c>
-      <c r="C9" s="7">
-        <f>IF(AND(D9="Sim",E9&gt;0,F9=E9,G9&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -680,9 +680,10 @@
           <t>Giovana Almeida Alves</t>
         </is>
       </c>
-      <c r="C10" s="7">
-        <f>IF(AND(D10="Sim",E10&gt;0,F10=E10,G10&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
@@ -721,9 +722,10 @@
           <t>Guilherme Melo Santos</t>
         </is>
       </c>
-      <c r="C11" s="7">
-        <f>IF(AND(D11="Sim",E11&gt;0,F11=E11,G11&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
@@ -762,9 +764,10 @@
           <t>Helo Andrade</t>
         </is>
       </c>
-      <c r="C12" s="7">
-        <f>IF(AND(D12="Sim",E12&gt;0,F12=E12,G12&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
@@ -799,9 +802,10 @@
           <t>Isabelly Oliveira</t>
         </is>
       </c>
-      <c r="C13" s="7">
-        <f>IF(AND(D13="Sim",E13&gt;0,F13=E13,G13&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
@@ -840,9 +844,10 @@
           <t>Miguel Souza Flor Dos Santos</t>
         </is>
       </c>
-      <c r="C14" s="7">
-        <f>IF(AND(D14="Sim",E14&gt;0,F14=E14,G14&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
@@ -877,9 +882,10 @@
           <t>Pedro Henrique Caraça</t>
         </is>
       </c>
-      <c r="C15" s="7">
-        <f>IF(AND(D15="Sim",E15&gt;0,F15=E15,G15&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
@@ -914,9 +920,10 @@
           <t>Ramon</t>
         </is>
       </c>
-      <c r="C16" s="7">
-        <f>IF(AND(D16="Sim",E16&gt;0,F16=E16,G16&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
@@ -955,9 +962,10 @@
           <t>Thiago Silva Bispo</t>
         </is>
       </c>
-      <c r="C17" s="7">
-        <f>IF(AND(D17="Sim",E17&gt;0,F17=E17,G17&gt;0),"Concluído","Pendente")</f>
-        <v/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Esther: capa, 6 fotos com versículo e louvor na Mensagem (falta áudio dos pais)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/controle.xlsx
+++ b/controle.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Controle'!$A$7:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Controle'!$A$8:$J$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -111,7 +111,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -123,6 +123,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FBEBDD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF6D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -488,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -530,116 +537,84 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>Parciais</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t>Pendentes</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="B6" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Nome completo</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Capa</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Fotos</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Versículos</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Áudios</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Link da página</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Link do QR code</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Catarina</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Catarina</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=catarina</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/catarina.png</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Esther</t>
+          <t>Catarina</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Esther Caraça</t>
+          <t>Catarina</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -653,7 +628,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>0</v>
@@ -661,28 +636,32 @@
       <c r="G9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Ainda não está no site</t>
-        </is>
-      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=catarina</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/catarina.png</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Giovana</t>
+          <t>Esther</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Giovana Almeida Alves</t>
+          <t>Esther Caraça</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Concluído</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -691,35 +670,39 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=giovana</t>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=esther</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/giovana.png</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr"/>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/esther.png</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Falta: áudio dos pais</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Guilherme</t>
+          <t>Giovana</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Guilherme Melo Santos</t>
+          <t>Giovana Almeida Alves</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -739,16 +722,16 @@
         <v>4</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=guilherme</t>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=giovana</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/guilherme.png</t>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/giovana.png</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr"/>
@@ -756,130 +739,134 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Helo</t>
+          <t>Guilherme</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Helo Andrade</t>
+          <t>Guilherme Melo Santos</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Ainda não está no site</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=guilherme</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/guilherme.png</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Isabelly</t>
+          <t>Helo</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Isabelly Oliveira</t>
+          <t>Helo Andrade</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Concluído</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=isabelly</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/isabelly.png</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Ainda não está no site</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Isabelly</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Miguel Souza Flor Dos Santos</t>
+          <t>Isabelly Oliveira</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6" t="inlineStr"/>
-      <c r="I14" s="6" t="inlineStr"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>Ainda não está no site</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=isabelly</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/isabelly.png</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Pedro</t>
+          <t>Miguel</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Pedro Henrique Caraça</t>
+          <t>Miguel Souza Flor Dos Santos</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -912,104 +899,147 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Ramon</t>
+          <t>Pedro</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Ramon</t>
+          <t>Pedro Henrique Caraça</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Concluído</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=ramon</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/ramon.png</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Ainda não está no site</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>Ramon</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Ramon</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=ramon</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/ramon.png</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
           <t>Thiago</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Thiago Silva Bispo</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="E17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="E18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Ainda não está no site</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:J17"/>
-  <conditionalFormatting sqref="A8:J17">
+  <autoFilter ref="A8:J18"/>
+  <conditionalFormatting sqref="A9:J18">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$C8="Concluído"</formula>
+      <formula>$C9="Concluído"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$C8="Pendente"</formula>
+      <formula>$C9="Pendente"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>$C9="Parcial"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pedro: capa sem cortar Jesus, 6 fotos com versículo e louvor na Mensagem (falta áudio dos pais)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/controle.xlsx
+++ b/controle.xlsx
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -909,28 +909,36 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="6" t="inlineStr"/>
-      <c r="I16" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/?id=pedro</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>https://olvlucasn.github.io/lembrancinha-igreja/qrcodes/pedro.png</t>
+        </is>
+      </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Ainda não está no site</t>
+          <t>Falta: áudio dos pais</t>
         </is>
       </c>
     </row>
@@ -1038,8 +1046,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>